<commit_message>
made a lot of changes presenting tomorrow
</commit_message>
<xml_diff>
--- a/information for modeling/travtiove system model .xlsx
+++ b/information for modeling/travtiove system model .xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muizz_1/Documents/information for modeling/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muizz_1/Documents/E27-Tractive-system-MATLAB-model-/information for modeling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C63B85B-BC3F-144B-A41F-EB627A5D1C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F89CFF-D0C2-4141-AA62-3F730EB060F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1400" yWindow="1240" windowWidth="28040" windowHeight="17180" activeTab="5" xr2:uid="{0FACE01F-734A-5E49-A078-B14114F26C95}"/>
+    <workbookView xWindow="1400" yWindow="1240" windowWidth="28040" windowHeight="17180" activeTab="3" xr2:uid="{0FACE01F-734A-5E49-A078-B14114F26C95}"/>
   </bookViews>
   <sheets>
     <sheet name="Accumalator grpah" sheetId="1" r:id="rId1"/>

</xml_diff>